<commit_message>
data: upsert 2022Q1 (update_quarter.py)
</commit_message>
<xml_diff>
--- a/data/再保偿付能力2023Q2-0901.xlsx
+++ b/data/再保偿付能力2023Q2-0901.xlsx
@@ -1544,10 +1544,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4.2378</v>
+        <v>4.237774</v>
       </c>
       <c r="D18" t="n">
-        <v>4.2378</v>
+        <v>4.237774</v>
       </c>
       <c r="E18" t="n">
         <v>6021001</v>

</xml_diff>